<commit_message>
Added readme to sample input
</commit_message>
<xml_diff>
--- a/sample_input.xlsx
+++ b/sample_input.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicolls/proj/eleceng_matlab/ilp_thesisalloc/2025s/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicolls/proj/eleceng/ilpalloc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E11C3FF-3F95-4140-B400-16AACD65F4C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92E8649-889A-CC44-8D9D-2C9A0E74F788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="19400" windowHeight="11480" activeTab="2" xr2:uid="{B85E0B53-F2B5-4C6A-A8EC-B81D8DF7DA2F}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="19400" windowHeight="11480" xr2:uid="{B85E0B53-F2B5-4C6A-A8EC-B81D8DF7DA2F}"/>
   </bookViews>
   <sheets>
-    <sheet name="choices" sheetId="1" r:id="rId1"/>
-    <sheet name="limits" sheetId="2" r:id="rId2"/>
-    <sheet name="scores" sheetId="3" r:id="rId3"/>
+    <sheet name="README" sheetId="4" r:id="rId1"/>
+    <sheet name="choices" sheetId="1" r:id="rId2"/>
+    <sheet name="limits" sheetId="2" r:id="rId3"/>
+    <sheet name="scores" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="354">
   <si>
     <t>WLTRON002</t>
   </si>
@@ -989,6 +990,117 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>README: Input File Format for Student Project Allocation</t>
+  </si>
+  <si>
+    <t>This Excel file is used by the ilpalloc.py script to allocate student projects based on preferences, supervisor limits, and scoring weights. The script solves an integer linear program (ILP) to assign students to projects fairly.</t>
+  </si>
+  <si>
+    <t>The file must contain exactly three sheets: 'choices', 'limits', and 'scores'. Below is a detailed description of each sheet's purpose and required format. If any sheet is missing or malformed, the script will raise an error.</t>
+  </si>
+  <si>
+    <t>1. 'choices' Sheet: Student Preferences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Purpose: Lists each student's project preferences. The script uses this to build the assignment constraints, prioritizing higher-ranked choices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Format:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - First column: "Student No" (unique identifier for each student, e.g., student ID or name).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Subsequent columns: "Topic ID Choice 1", "Topic ID Choice 2", ..., "Topic ID Choice N" (where N is the number of choices, up to the maximum in the data).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Each cell contains a project code (e.g., "ABC123" for a supervisor's project). Leave blank if no preference for that rank.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Project codes should follow a pattern: uppercase letters for supervisor (e.g., "ABC" for supervisor ABC), optionally followed by lowercase for self-proposed projects.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Example: See the 'choices' sheet in this file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Notes:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - The number of choice columns determines the maximum preferences considered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Self-proposed projects (codes with lowercase) are handled specially.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Ensure no duplicates in student IDs.</t>
+  </si>
+  <si>
+    <t>2. 'limits' Sheet: Supervisor Capacity Limits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Purpose: Defines the maximum number of students each supervisor can oversee. The script enforces these as hard constraints in the ILP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Two columns: "Supervisor" and "Max".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - "Supervisor": Short code (uppercase letters, e.g., "ABC") matching the prefix in project codes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - "Max": Integer limit (e.g., 5). Use "*" in the Supervisor column for a default limit applied to all supervisors without specific limits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Example: See the 'limits' sheet in this file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - The default ("*") is used if a supervisor isn't listed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Limits must be positive integers.</t>
+  </si>
+  <si>
+    <t>3. 'scores' Sheet: Preference Weights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Purpose: Assigns scores to each choice rank (e.g., first choice gets a higher score). The ILP minimizes the total "cost" based on these scores, so higher scores mean better preferences.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Two columns: "Choice" and "Score".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - "Choice": Integer rank (1 for first choice, 2 for second, etc.).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - "Score": Float value (e.g., 10.0 for first choice, decreasing for lower ranks).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Example: See the 'scores' sheet in this file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - Scores should decrease with rank (higher number = better).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     - The script uses these to weight preferences in the objective function.</t>
+  </si>
+  <si>
+    <t>General Notes:</t>
+  </si>
+  <si>
+    <t>- File Name: Save as .xlsx (e.g., sample_input.xlsx). Pass the path as an argument to the script: python ilpalloc.py path/to/file.xlsx.</t>
+  </si>
+  <si>
+    <t>- Output: The script generates file_results.xlsx with 'allocations' and 'unallocated' sheets.</t>
+  </si>
+  <si>
+    <t>- Requirements: Ensure pandas, numpy, and pulp are installed. The script uses CBC or HiGHS solver (install via conda if needed).</t>
+  </si>
+  <si>
+    <t>- Validation: The script checks for missing data and raises errors for invalid formats.</t>
+  </si>
+  <si>
+    <t>- Customization: Adjust scores/limits based on your needs. For large datasets, solver performance may vary.</t>
   </si>
 </sst>
 </file>
@@ -1403,6 +1515,221 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EE03BC7-D2AE-B545-9C76-C3A111AEEC6A}">
+  <dimension ref="A1:A47"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>353</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5D1384-99BD-4D3F-9275-0834FCD7DDB0}">
   <dimension ref="A1:G106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3863,7 +4190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3DCFFDE-D4EB-164B-BF92-4C3D5FF5A821}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3937,7 +4264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0010CE6B-C5FD-4144-BFAB-819BCB8A9B09}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>